<commit_message>
Finalización de simulador, realización de simulaciones y estructuración del proyecto.
</commit_message>
<xml_diff>
--- a/src/data/raw/meals/Meals.xlsx
+++ b/src/data/raw/meals/Meals.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF44A92B-F229-4038-B9E4-CBC4D487B74B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{751732AA-2890-4D02-942D-F4B36FE76A73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{815E471D-FB27-4CE8-A9B5-FEF30EA8CD57}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$V$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$V$36</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="90">
   <si>
     <t>Comida</t>
   </si>
@@ -197,9 +197,6 @@
     <t>Costillas de Cerdo BBQ</t>
   </si>
   <si>
-    <t>Rollitos Primavera</t>
-  </si>
-  <si>
     <t>Blue Cheese</t>
   </si>
   <si>
@@ -305,13 +302,13 @@
     <t>game (deer, venison)</t>
   </si>
   <si>
-    <t>rich fish (salmon, tuna, etc)</t>
-  </si>
-  <si>
     <t>Game (deer, venison)</t>
   </si>
   <si>
     <t>Rich Fish (salmon, tuna etc)</t>
+  </si>
+  <si>
+    <t>rich fish (salmon, tuna etc)</t>
   </si>
 </sst>
 </file>
@@ -683,7 +680,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{788D91E9-4975-43F6-A96D-CD05AC054CF1}">
-  <dimension ref="A1:V53"/>
+  <dimension ref="A1:V52"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.28515625" bestFit="1" customWidth="1"/>
@@ -713,7 +710,7 @@
         <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I1" t="s">
         <v>7</v>
@@ -743,7 +740,7 @@
         <v>15</v>
       </c>
       <c r="R1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="S1" t="s">
         <v>16</v>
@@ -828,13 +825,13 @@
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>52</v>
+        <v>76</v>
       </c>
       <c r="B3" t="s">
         <v>44</v>
       </c>
       <c r="C3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -888,21 +885,21 @@
         <v>0</v>
       </c>
       <c r="U3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>77</v>
+        <v>59</v>
       </c>
       <c r="B4" t="s">
         <v>44</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -914,7 +911,7 @@
         <v>0</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H4">
         <v>0</v>
@@ -932,7 +929,7 @@
         <v>0</v>
       </c>
       <c r="M4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N4">
         <v>0</v>
@@ -964,25 +961,25 @@
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B5" t="s">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="C5">
         <v>0</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5">
         <v>0</v>
       </c>
       <c r="G5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H5">
         <v>0</v>
@@ -1000,7 +997,7 @@
         <v>0</v>
       </c>
       <c r="M5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N5">
         <v>0</v>
@@ -1024,7 +1021,7 @@
         <v>0</v>
       </c>
       <c r="U5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V5">
         <v>0</v>
@@ -1032,7 +1029,7 @@
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="B6" t="s">
         <v>23</v>
@@ -1071,7 +1068,7 @@
         <v>0</v>
       </c>
       <c r="N6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O6">
         <v>0</v>
@@ -1092,7 +1089,7 @@
         <v>0</v>
       </c>
       <c r="U6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V6">
         <v>0</v>
@@ -1100,7 +1097,7 @@
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="B7" t="s">
         <v>23</v>
@@ -1139,7 +1136,7 @@
         <v>0</v>
       </c>
       <c r="N7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O7">
         <v>0</v>
@@ -1168,7 +1165,7 @@
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="B8" t="s">
         <v>23</v>
@@ -1236,7 +1233,7 @@
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>76</v>
+        <v>56</v>
       </c>
       <c r="B9" t="s">
         <v>23</v>
@@ -1272,7 +1269,7 @@
         <v>0</v>
       </c>
       <c r="M9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N9">
         <v>0</v>
@@ -1304,7 +1301,7 @@
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="B10" t="s">
         <v>23</v>
@@ -1340,7 +1337,7 @@
         <v>0</v>
       </c>
       <c r="M10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N10">
         <v>0</v>
@@ -1349,7 +1346,7 @@
         <v>0</v>
       </c>
       <c r="P10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q10">
         <v>0</v>
@@ -1361,7 +1358,7 @@
         <v>0</v>
       </c>
       <c r="T10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U10">
         <v>0</v>
@@ -1372,7 +1369,7 @@
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="B11" t="s">
         <v>23</v>
@@ -1417,7 +1414,7 @@
         <v>0</v>
       </c>
       <c r="P11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q11">
         <v>0</v>
@@ -1440,7 +1437,7 @@
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="B12" t="s">
         <v>23</v>
@@ -1497,7 +1494,7 @@
         <v>0</v>
       </c>
       <c r="T12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U12">
         <v>0</v>
@@ -1508,7 +1505,7 @@
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="B13" t="s">
         <v>23</v>
@@ -1544,7 +1541,7 @@
         <v>0</v>
       </c>
       <c r="M13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N13">
         <v>0</v>
@@ -1612,7 +1609,7 @@
         <v>0</v>
       </c>
       <c r="M14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N14">
         <v>0</v>
@@ -1644,10 +1641,10 @@
     </row>
     <row r="15" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="B15" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C15">
         <v>0</v>
@@ -1656,10 +1653,10 @@
         <v>0</v>
       </c>
       <c r="E15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G15">
         <v>0</v>
@@ -1686,7 +1683,7 @@
         <v>0</v>
       </c>
       <c r="O15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P15">
         <v>0</v>
@@ -1712,10 +1709,10 @@
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C16">
         <v>0</v>
@@ -1754,7 +1751,7 @@
         <v>0</v>
       </c>
       <c r="O16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P16">
         <v>0</v>
@@ -1780,16 +1777,16 @@
     </row>
     <row r="17" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>78</v>
+        <v>25</v>
       </c>
       <c r="B17" t="s">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="C17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E17">
         <v>0</v>
@@ -1798,13 +1795,13 @@
         <v>1</v>
       </c>
       <c r="G17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H17">
         <v>0</v>
       </c>
       <c r="I17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J17">
         <v>0</v>
@@ -1813,10 +1810,10 @@
         <v>0</v>
       </c>
       <c r="L17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N17">
         <v>0</v>
@@ -1848,31 +1845,31 @@
     </row>
     <row r="18" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="B18" t="s">
-        <v>26</v>
+        <v>87</v>
       </c>
       <c r="C18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E18">
         <v>0</v>
       </c>
       <c r="F18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J18">
         <v>0</v>
@@ -1881,10 +1878,10 @@
         <v>0</v>
       </c>
       <c r="L18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N18">
         <v>0</v>
@@ -1916,10 +1913,10 @@
     </row>
     <row r="19" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="B19" t="s">
-        <v>89</v>
+        <v>28</v>
       </c>
       <c r="C19">
         <v>0</v>
@@ -1937,13 +1934,13 @@
         <v>0</v>
       </c>
       <c r="H19">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I19">
         <v>0</v>
       </c>
       <c r="J19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K19">
         <v>0</v>
@@ -1984,10 +1981,10 @@
     </row>
     <row r="20" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
       <c r="B20" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="C20">
         <v>0</v>
@@ -2011,7 +2008,7 @@
         <v>0</v>
       </c>
       <c r="J20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K20">
         <v>0</v>
@@ -2035,7 +2032,7 @@
         <v>0</v>
       </c>
       <c r="R20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S20">
         <v>0</v>
@@ -2052,10 +2049,10 @@
     </row>
     <row r="21" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="B21" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="C21">
         <v>0</v>
@@ -2085,10 +2082,10 @@
         <v>0</v>
       </c>
       <c r="L21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N21">
         <v>0</v>
@@ -2103,7 +2100,7 @@
         <v>0</v>
       </c>
       <c r="R21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S21">
         <v>0</v>
@@ -2120,10 +2117,10 @@
     </row>
     <row r="22" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>46</v>
+        <v>70</v>
       </c>
       <c r="B22" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="C22">
         <v>0</v>
@@ -2138,7 +2135,7 @@
         <v>0</v>
       </c>
       <c r="G22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H22">
         <v>0</v>
@@ -2153,7 +2150,7 @@
         <v>0</v>
       </c>
       <c r="L22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M22">
         <v>1</v>
@@ -2183,15 +2180,15 @@
         <v>0</v>
       </c>
       <c r="V22">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>71</v>
+        <v>29</v>
       </c>
       <c r="B23" t="s">
-        <v>73</v>
+        <v>30</v>
       </c>
       <c r="C23">
         <v>0</v>
@@ -2206,7 +2203,7 @@
         <v>0</v>
       </c>
       <c r="G23">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H23">
         <v>0</v>
@@ -2224,10 +2221,10 @@
         <v>0</v>
       </c>
       <c r="M23">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O23">
         <v>0</v>
@@ -2251,15 +2248,15 @@
         <v>0</v>
       </c>
       <c r="V23">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="B24" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C24">
         <v>0</v>
@@ -2274,7 +2271,7 @@
         <v>0</v>
       </c>
       <c r="G24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H24">
         <v>0</v>
@@ -2292,13 +2289,13 @@
         <v>0</v>
       </c>
       <c r="M24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N24">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P24">
         <v>0</v>
@@ -2319,7 +2316,7 @@
         <v>0</v>
       </c>
       <c r="V24">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:22" x14ac:dyDescent="0.25">
@@ -2342,7 +2339,7 @@
         <v>0</v>
       </c>
       <c r="G25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H25">
         <v>0</v>
@@ -2387,12 +2384,12 @@
         <v>0</v>
       </c>
       <c r="V25">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>55</v>
+        <v>82</v>
       </c>
       <c r="B26" t="s">
         <v>20</v>
@@ -2428,7 +2425,7 @@
         <v>0</v>
       </c>
       <c r="M26">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N26">
         <v>0</v>
@@ -2455,12 +2452,12 @@
         <v>0</v>
       </c>
       <c r="V26">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="B27" t="s">
         <v>20</v>
@@ -2523,15 +2520,15 @@
         <v>0</v>
       </c>
       <c r="V27">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>75</v>
+        <v>42</v>
       </c>
       <c r="B28" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="C28">
         <v>0</v>
@@ -2570,10 +2567,10 @@
         <v>0</v>
       </c>
       <c r="O28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P28">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q28">
         <v>0</v>
@@ -2585,18 +2582,18 @@
         <v>0</v>
       </c>
       <c r="T28">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U28">
         <v>0</v>
       </c>
       <c r="V28">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B29" t="s">
         <v>32</v>
@@ -2614,7 +2611,7 @@
         <v>0</v>
       </c>
       <c r="G29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H29">
         <v>0</v>
@@ -2653,7 +2650,7 @@
         <v>0</v>
       </c>
       <c r="T29">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U29">
         <v>0</v>
@@ -2664,7 +2661,7 @@
     </row>
     <row r="30" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B30" t="s">
         <v>32</v>
@@ -2682,7 +2679,7 @@
         <v>0</v>
       </c>
       <c r="G30">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H30">
         <v>0</v>
@@ -2721,7 +2718,7 @@
         <v>0</v>
       </c>
       <c r="T30">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U30">
         <v>0</v>
@@ -2732,7 +2729,7 @@
     </row>
     <row r="31" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>51</v>
+        <v>67</v>
       </c>
       <c r="B31" t="s">
         <v>32</v>
@@ -2768,7 +2765,7 @@
         <v>0</v>
       </c>
       <c r="M31">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N31">
         <v>0</v>
@@ -2789,7 +2786,7 @@
         <v>0</v>
       </c>
       <c r="T31">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U31">
         <v>0</v>
@@ -2800,7 +2797,7 @@
     </row>
     <row r="32" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>68</v>
+        <v>31</v>
       </c>
       <c r="B32" t="s">
         <v>32</v>
@@ -2836,7 +2833,7 @@
         <v>0</v>
       </c>
       <c r="M32">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N32">
         <v>0</v>
@@ -2868,10 +2865,10 @@
     </row>
     <row r="33" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>69</v>
       </c>
       <c r="B33" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="C33">
         <v>0</v>
@@ -2913,10 +2910,10 @@
         <v>0</v>
       </c>
       <c r="P33">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q33">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R33">
         <v>0</v>
@@ -2936,7 +2933,7 @@
     </row>
     <row r="34" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="B34" t="s">
         <v>22</v>
@@ -3004,7 +3001,7 @@
     </row>
     <row r="35" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>66</v>
+        <v>49</v>
       </c>
       <c r="B35" t="s">
         <v>22</v>
@@ -3040,7 +3037,7 @@
         <v>0</v>
       </c>
       <c r="M35">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N35">
         <v>0</v>
@@ -3072,7 +3069,7 @@
     </row>
     <row r="36" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="B36" t="s">
         <v>22</v>
@@ -3108,7 +3105,7 @@
         <v>0</v>
       </c>
       <c r="M36">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N36">
         <v>0</v>
@@ -3129,7 +3126,7 @@
         <v>0</v>
       </c>
       <c r="T36">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U36">
         <v>0</v>
@@ -3140,7 +3137,7 @@
     </row>
     <row r="37" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>59</v>
+        <v>78</v>
       </c>
       <c r="B37" t="s">
         <v>22</v>
@@ -3197,7 +3194,7 @@
         <v>0</v>
       </c>
       <c r="T37">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U37">
         <v>0</v>
@@ -3208,10 +3205,10 @@
     </row>
     <row r="38" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>79</v>
+        <v>21</v>
       </c>
       <c r="B38" t="s">
-        <v>22</v>
+        <v>88</v>
       </c>
       <c r="C38">
         <v>0</v>
@@ -3256,10 +3253,10 @@
         <v>0</v>
       </c>
       <c r="Q38">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R38">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S38">
         <v>0</v>
@@ -3276,10 +3273,10 @@
     </row>
     <row r="39" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="B39" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C39">
         <v>0</v>
@@ -3344,16 +3341,16 @@
     </row>
     <row r="40" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="B40" t="s">
-        <v>90</v>
+        <v>34</v>
       </c>
       <c r="C40">
         <v>0</v>
       </c>
       <c r="D40">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E40">
         <v>0</v>
@@ -3374,7 +3371,7 @@
         <v>0</v>
       </c>
       <c r="K40">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L40">
         <v>0</v>
@@ -3395,10 +3392,10 @@
         <v>0</v>
       </c>
       <c r="R40">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S40">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T40">
         <v>0</v>
@@ -3412,7 +3409,7 @@
     </row>
     <row r="41" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="B41" t="s">
         <v>34</v>
@@ -3442,7 +3439,7 @@
         <v>0</v>
       </c>
       <c r="K41">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L41">
         <v>0</v>
@@ -3480,13 +3477,13 @@
     </row>
     <row r="42" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="B42" t="s">
         <v>34</v>
       </c>
       <c r="C42">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D42">
         <v>1</v>
@@ -3548,16 +3545,16 @@
     </row>
     <row r="43" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B43" t="s">
         <v>34</v>
       </c>
       <c r="C43">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D43">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E43">
         <v>0</v>
@@ -3616,10 +3613,10 @@
     </row>
     <row r="44" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>39</v>
+        <v>83</v>
       </c>
       <c r="B44" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="C44">
         <v>0</v>
@@ -3670,13 +3667,13 @@
         <v>0</v>
       </c>
       <c r="S44">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T44">
         <v>0</v>
       </c>
       <c r="U44">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V44">
         <v>0</v>
@@ -3684,10 +3681,10 @@
     </row>
     <row r="45" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="B45" t="s">
-        <v>41</v>
+        <v>24</v>
       </c>
       <c r="C45">
         <v>0</v>
@@ -3744,15 +3741,15 @@
         <v>0</v>
       </c>
       <c r="U45">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V45">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>72</v>
+        <v>55</v>
       </c>
       <c r="B46" t="s">
         <v>24</v>
@@ -3820,7 +3817,7 @@
     </row>
     <row r="47" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="B47" t="s">
         <v>24</v>
@@ -3888,7 +3885,7 @@
     </row>
     <row r="48" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>48</v>
+        <v>62</v>
       </c>
       <c r="B48" t="s">
         <v>24</v>
@@ -3924,7 +3921,7 @@
         <v>0</v>
       </c>
       <c r="M48">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N48">
         <v>0</v>
@@ -3956,7 +3953,7 @@
     </row>
     <row r="49" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>63</v>
+        <v>37</v>
       </c>
       <c r="B49" t="s">
         <v>24</v>
@@ -3965,7 +3962,7 @@
         <v>0</v>
       </c>
       <c r="D49">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E49">
         <v>0</v>
@@ -3989,10 +3986,10 @@
         <v>0</v>
       </c>
       <c r="L49">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M49">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N49">
         <v>0</v>
@@ -4024,7 +4021,7 @@
     </row>
     <row r="50" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>37</v>
+        <v>84</v>
       </c>
       <c r="B50" t="s">
         <v>24</v>
@@ -4092,7 +4089,7 @@
     </row>
     <row r="51" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>85</v>
+        <v>61</v>
       </c>
       <c r="B51" t="s">
         <v>24</v>
@@ -4101,7 +4098,7 @@
         <v>0</v>
       </c>
       <c r="D51">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E51">
         <v>0</v>
@@ -4125,10 +4122,10 @@
         <v>0</v>
       </c>
       <c r="L51">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M51">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N51">
         <v>0</v>
@@ -4160,7 +4157,7 @@
     </row>
     <row r="52" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="B52" t="s">
         <v>24</v>
@@ -4169,7 +4166,7 @@
         <v>0</v>
       </c>
       <c r="D52">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E52">
         <v>0</v>
@@ -4196,7 +4193,7 @@
         <v>0</v>
       </c>
       <c r="M52">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N52">
         <v>0</v>
@@ -4226,76 +4223,8 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>86</v>
-      </c>
-      <c r="B53" t="s">
-        <v>24</v>
-      </c>
-      <c r="C53">
-        <v>0</v>
-      </c>
-      <c r="D53">
-        <v>1</v>
-      </c>
-      <c r="E53">
-        <v>0</v>
-      </c>
-      <c r="F53">
-        <v>0</v>
-      </c>
-      <c r="G53">
-        <v>0</v>
-      </c>
-      <c r="H53">
-        <v>0</v>
-      </c>
-      <c r="I53">
-        <v>0</v>
-      </c>
-      <c r="J53">
-        <v>0</v>
-      </c>
-      <c r="K53">
-        <v>0</v>
-      </c>
-      <c r="L53">
-        <v>0</v>
-      </c>
-      <c r="M53">
-        <v>0</v>
-      </c>
-      <c r="N53">
-        <v>0</v>
-      </c>
-      <c r="O53">
-        <v>0</v>
-      </c>
-      <c r="P53">
-        <v>0</v>
-      </c>
-      <c r="Q53">
-        <v>0</v>
-      </c>
-      <c r="R53">
-        <v>0</v>
-      </c>
-      <c r="S53">
-        <v>0</v>
-      </c>
-      <c r="T53">
-        <v>0</v>
-      </c>
-      <c r="U53">
-        <v>0</v>
-      </c>
-      <c r="V53">
-        <v>1</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:V37" xr:uid="{788D91E9-4975-43F6-A96D-CD05AC054CF1}"/>
+  <autoFilter ref="A1:V36" xr:uid="{788D91E9-4975-43F6-A96D-CD05AC054CF1}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>